<commit_message>
docs: refine order flow review and customer QA
</commit_message>
<xml_diff>
--- a/doc/QA khách hàng v1.xlsx
+++ b/doc/QA khách hàng v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\zootopbear-usecase\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92698B6F-CBC7-44B5-B083-6C2E33E00F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DC94B4-67AA-4AE2-B934-49A9756792EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chức năng mong muốn" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,11 @@
     <sheet name="thông tin account nhà cung cấp" sheetId="5" r:id="rId5"/>
     <sheet name="QA ngày 21-07" sheetId="6" r:id="rId6"/>
     <sheet name="Xác nhận role 21-07" sheetId="7" r:id="rId7"/>
+    <sheet name="QA_order_flow" sheetId="8" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">QA_order_flow!$A$1:$F$1</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -31,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="766">
   <si>
     <t>STT</t>
   </si>
@@ -2266,12 +2270,156 @@
   <si>
     <t>Em muốn có thêm chức năng tạo ticket như bên Simple hub, tức là khách nếu có vấn đề cần sửa với đơn hàng sẽ tạo ticket trên hệ thống, sau đó ticket và vấn đề đó sẽ nhảy API đến xưởng tương ứng, a có thể vào Simple hub xem chức năng TICKET ĐÓ</t>
   </si>
+  <si>
+    <t>Câu hỏi gửi khách</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại để khách xác nhận/sửa</t>
+  </si>
+  <si>
+    <t>Khách trả lời</t>
+  </si>
+  <si>
+    <t>Luồng tổng quan</t>
+  </si>
+  <si>
+    <t>Hiện tại seller gửi danh sách đơn cho Zootop bằng file Excel/list đơn, sau đó nhân viên Zootop xử lý tiếp trên file nội bộ. Cách hiểu này có đúng với luồng đang chạy không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: seller chưa thao tác trực tiếp trên hệ thống Zootop; seller gửi dữ liệu đơn, Zootop kiểm tra - tính tiền - đưa đơn sang xưởng.</t>
+  </si>
+  <si>
+    <t>Cấu trúc đơn</t>
+  </si>
+  <si>
+    <t>Nếu một đơn có nhiều sản phẩm, hiện tại file sẽ có nhiều dòng cùng một mã đơn, mỗi dòng là một sản phẩm/item. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: Order ID là mã dùng để gom nhiều dòng thành cùng một đơn khi tính tiền và theo dõi.</t>
+  </si>
+  <si>
+    <t>Thông tin bắt buộc</t>
+  </si>
+  <si>
+    <t>Một đơn trước khi gửi xưởng cần có: thông tin người nhận, mã hàng/phiên bản sản phẩm, số lượng, link thiết kế/mockup, hình thức giao hàng hoặc label nếu có. Có thiếu thông tin quan trọng nào không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: đây là nhóm dữ liệu tối thiểu để xưởng có thể sản xuất và giao hàng.</t>
+  </si>
+  <si>
+    <t>Kiểm tra dữ liệu</t>
+  </si>
+  <si>
+    <t>Trước khi đưa đơn sang xưởng, nhân viên Zootop đang kiểm tra lỗi như thiếu địa chỉ, sai mã hàng, link thiết kế không mở được, thiếu mockup hoặc file trước/sau bị lệch. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: các đơn lỗi chưa đi xưởng ngay mà được tách ra để xử lý riêng.</t>
+  </si>
+  <si>
+    <t>Nhóm sản phẩm</t>
+  </si>
+  <si>
+    <t>Các nhóm như Home Decor, Mug, Accessories/Home Living, Gildan/Apparel đang có cách xử lý và công thức tính tiền riêng. Web mới cần giữ logic riêng theo từng nhóm sản phẩm, đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: không thể dùng một công thức chung cho toàn bộ sản phẩm.</t>
+  </si>
+  <si>
+    <t>Tính tiền</t>
+  </si>
+  <si>
+    <t>Tổng tiền đơn hiện được tính từ tiền sản phẩm, phí ship hoặc phí label, phí item thêm và có thể có phí in thêm với áo. Cách hiểu này có đúng với Excel hiện tại không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: nhiều dòng cùng mã đơn được gom lại; phí ship/label thường không tính lặp trên mọi dòng.</t>
+  </si>
+  <si>
+    <t>Giá seller và giá xưởng</t>
+  </si>
+  <si>
+    <t>Zootop có một giá tính cho seller, còn giá/cost khi tạo đơn trên từng xưởng là một lớp giá khác dùng để đối soát nội bộ. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: seller không nhất thiết nhìn thấy giá vốn của xưởng.</t>
+  </si>
+  <si>
+    <t>Tìm xưởng sản xuất</t>
+  </si>
+  <si>
+    <t>Sau khi biết mã hàng/phiên bản sản phẩm, Zootop tra bảng mapping để biết đơn sẽ đi sang xưởng nào, ví dụ PrintBelle hoặc các mã nội bộ như 415/922. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: mã hàng không chỉ dùng để tính giá mà còn dùng để chọn xưởng xử lý.</t>
+  </si>
+  <si>
+    <t>Đẩy đơn sang xưởng</t>
+  </si>
+  <si>
+    <t>Với đơn đã đủ dữ liệu và đã xác định được xưởng, nhân viên Zootop hiện tạo đơn trên nền tảng của xưởng bằng web/portal, upload file hoặc kết nối tự động tùy xưởng. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: mỗi xưởng có cách đưa đơn lên khác nhau; web mới cần mô phỏng hoặc tự động hóa dần phần này.</t>
+  </si>
+  <si>
+    <t>5 xưởng/nền tảng</t>
+  </si>
+  <si>
+    <t>Hiện các xưởng/nền tảng phía sau gồm FlashShip, SimplePrint, PrintBelle, ART ADD và Snap Ecom. Có xưởng nào đang dùng cho đơn hiện tại nhưng chưa nằm trong danh sách này không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: đây là 5 nơi Zootop dùng để sản xuất/fulfill đơn cho seller.</t>
+  </si>
+  <si>
+    <t>Mã đơn của xưởng</t>
+  </si>
+  <si>
+    <t>Sau khi đơn được tạo trên xưởng, xưởng có thể sinh mã đơn/mã hàng riêng. Zootop cần lưu lại các mã này để tra cứu, đối soát và xử lý support. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: mã đơn seller/Zootop và mã đơn của xưởng là hai loại mã khác nhau.</t>
+  </si>
+  <si>
+    <t>Mã vận đơn</t>
+  </si>
+  <si>
+    <t>Sau khi xưởng ship hàng, Zootop nhận hoặc export mã vận đơn, hãng vận chuyển và trạng thái giao hàng rồi cập nhật lại vào file theo dõi. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: mã vận đơn là dữ liệu trả về sau khi xưởng đã xử lý/gửi hàng.</t>
+  </si>
+  <si>
+    <t>Đối chiếu tracking</t>
+  </si>
+  <si>
+    <t>Khi cập nhật mã vận đơn, Zootop đối chiếu bằng mã đơn, mã hàng hoặc mã đơn của xưởng để gắn đúng tracking vào đúng đơn ban đầu. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: bước đối chiếu này giúp tránh nhầm tracking giữa các đơn hoặc giữa các seller.</t>
+  </si>
+  <si>
+    <t>Lỗi, gửi lại, hoàn tiền</t>
+  </si>
+  <si>
+    <t>Các trường hợp như lỗi thiết kế, lỗi import, giao sai, hàng lỗi, cần gửi lại hoặc hoàn tiền hiện đang được theo dõi riêng ở sheet Issue/Import lỗi. Web mới nên chuyển phần này thành luồng xử lý lỗi/ticket/refund/resend. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: đây là luồng phụ nhưng rất quan trọng, không chỉ là ghi chú đơn hàng.</t>
+  </si>
+  <si>
+    <t>Trạng thái seller nhìn thấy</t>
+  </si>
+  <si>
+    <t>Trên web mới, seller nên thấy trạng thái dễ hiểu như đang xử lý, đã gửi xưởng, đã có mã vận đơn, đang vận chuyển, đã giao, cần hỗ trợ; còn mã nội bộ của xưởng nên để Zootop xem. Cách hiểu này có đúng không?</t>
+  </si>
+  <si>
+    <t>Ý hiểu hiện tại: seller không cần nhìn các mã nội bộ như 415/922 hoặc mã SKU riêng của xưởng nếu không cần thiết.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2334,8 +2482,23 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2360,8 +2523,14 @@
         <bgColor rgb="FFCFE2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -2378,11 +2547,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2419,6 +2603,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -38314,4 +38504,284 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0EE2F93-602F-4102-84A7-D684AD688C35}">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="58.7109375" customWidth="1"/>
+    <col min="4" max="4" width="52.7109375" customWidth="1"/>
+    <col min="5" max="5" width="30.7109375" customWidth="1"/>
+    <col min="6" max="6" width="28.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>718</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>720</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="14">
+        <v>1</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>721</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>722</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+    </row>
+    <row r="3" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="14">
+        <v>2</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>724</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>725</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>726</v>
+      </c>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+    </row>
+    <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="14">
+        <v>3</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>727</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>728</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>729</v>
+      </c>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+    </row>
+    <row r="5" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="14">
+        <v>4</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>730</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>731</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>732</v>
+      </c>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+    </row>
+    <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="14">
+        <v>5</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>733</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>734</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>735</v>
+      </c>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+    </row>
+    <row r="7" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="14">
+        <v>6</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>736</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>737</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>738</v>
+      </c>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+    </row>
+    <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="14">
+        <v>7</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>739</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>740</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>741</v>
+      </c>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+    </row>
+    <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="14">
+        <v>8</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>742</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>743</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>744</v>
+      </c>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+    </row>
+    <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="14">
+        <v>9</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>745</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>746</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>747</v>
+      </c>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+    </row>
+    <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="14">
+        <v>10</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>748</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>749</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>750</v>
+      </c>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+    </row>
+    <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="14">
+        <v>11</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>751</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>752</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>753</v>
+      </c>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+    </row>
+    <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="14">
+        <v>12</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>754</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>755</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>756</v>
+      </c>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>757</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>758</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>759</v>
+      </c>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+    </row>
+    <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="14">
+        <v>14</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>760</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>761</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>762</v>
+      </c>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+    </row>
+    <row r="16" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="14">
+        <v>15</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>763</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>764</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>765</v>
+      </c>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{A0EE2F93-602F-4102-84A7-D684AD688C35}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>